<commit_message>
Lecture 9 practice set: lecture vocabulary in the sheet and the page
Atomic task, time spent, success criteria, verifier, verification type and
data replace the plain-English column names; the build-a-model column and
the pick step move to a later practice set.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/_plan/l09-template/verify-your-own-job-template.xlsx
+++ b/_plan/l09-template/verify-your-own-job-template.xlsx
@@ -451,7 +451,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I88"/>
+  <dimension ref="A1:H88"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="36" customWidth="1" min="1" max="1"/>
@@ -462,7 +462,6 @@
     <col width="14" customWidth="1" min="6" max="6"/>
     <col width="16" customWidth="1" min="7" max="7"/>
     <col width="14" customWidth="1" min="8" max="8"/>
-    <col width="13" customWidth="1" min="9" max="9"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -487,7 +486,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>My guess, before counting: share of tasks a rule or a judge can check</t>
+          <t>My guess, before counting: share of tasks that are verifiable</t>
         </is>
       </c>
       <c r="B3" s="4" t="n">
@@ -497,7 +496,7 @@
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>Tasks a rule or a judge can check</t>
+          <t>Verifiable tasks</t>
         </is>
       </c>
       <c r="B4" s="5">
@@ -508,7 +507,7 @@
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>Hours a rule or a judge can check</t>
+          <t>Verifiable time</t>
         </is>
       </c>
       <c r="B5" s="5">
@@ -519,7 +518,7 @@
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>Checkable, with past examples</t>
+          <t>Verifiable, and the data exists</t>
         </is>
       </c>
       <c r="B6" s="5">
@@ -530,20 +529,20 @@
     <row r="8" ht="66" customHeight="1">
       <c r="A8" s="6" t="inlineStr">
         <is>
-          <t>Task
+          <t>Atomic task
 (verb + what you produced)</t>
         </is>
       </c>
       <c r="B8" s="6" t="inlineStr">
         <is>
-          <t>Minutes
-last week</t>
+          <t>Time spent
+(minutes)</t>
         </is>
       </c>
       <c r="C8" s="6" t="inlineStr">
         <is>
-          <t>Done right when…
-(what must be true for it to count as done well)</t>
+          <t>Success criteria
+(what must be true for it to count as done)</t>
         </is>
       </c>
       <c r="D8" s="6" t="inlineStr">
@@ -554,30 +553,24 @@
       </c>
       <c r="E8" s="6" t="inlineStr">
         <is>
-          <t>Who or what checks it
+          <t>Verifier
 (a rule, or judge · signal · when)</t>
         </is>
       </c>
       <c r="F8" s="6" t="inlineStr">
         <is>
-          <t>Type</t>
+          <t>Verification type</t>
         </is>
       </c>
       <c r="G8" s="6" t="inlineStr">
         <is>
-          <t>Past examples
-(input + correct output)</t>
+          <t>Data
+(past input and output pairs)</t>
         </is>
       </c>
       <c r="H8" s="6" t="inlineStr">
         <is>
           <t>Bucket</t>
-        </is>
-      </c>
-      <c r="I8" s="6" t="inlineStr">
-        <is>
-          <t>Build a model for this?
-(pick one)</t>
         </is>
       </c>
     </row>
@@ -620,7 +613,6 @@
           <t>Automate</t>
         </is>
       </c>
-      <c r="I9" s="2" t="n"/>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
@@ -661,11 +653,6 @@
           <t>Augment</t>
         </is>
       </c>
-      <c r="I10" s="2" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
@@ -706,7 +693,6 @@
           <t>Automate</t>
         </is>
       </c>
-      <c r="I11" s="2" t="n"/>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
@@ -747,7 +733,6 @@
           <t>Automate</t>
         </is>
       </c>
-      <c r="I12" s="2" t="n"/>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
@@ -772,7 +757,6 @@
       <c r="F13" s="2" t="n"/>
       <c r="G13" s="2" t="n"/>
       <c r="H13" s="2" t="n"/>
-      <c r="I13" s="2" t="n"/>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
@@ -813,7 +797,6 @@
           <t>Augment</t>
         </is>
       </c>
-      <c r="I14" s="2" t="n"/>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
@@ -854,7 +837,6 @@
           <t>Augment</t>
         </is>
       </c>
-      <c r="I15" s="2" t="n"/>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
@@ -895,7 +877,6 @@
           <t>Augment</t>
         </is>
       </c>
-      <c r="I16" s="2" t="n"/>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
@@ -936,7 +917,6 @@
           <t>Human</t>
         </is>
       </c>
-      <c r="I17" s="2" t="n"/>
     </row>
     <row r="18">
       <c r="A18" s="2" t="n"/>
@@ -947,7 +927,6 @@
       <c r="F18" s="2" t="n"/>
       <c r="G18" s="2" t="n"/>
       <c r="H18" s="2" t="n"/>
-      <c r="I18" s="2" t="n"/>
     </row>
     <row r="19">
       <c r="A19" s="2" t="n"/>
@@ -958,7 +937,6 @@
       <c r="F19" s="2" t="n"/>
       <c r="G19" s="2" t="n"/>
       <c r="H19" s="2" t="n"/>
-      <c r="I19" s="2" t="n"/>
     </row>
     <row r="20">
       <c r="A20" s="2" t="n"/>
@@ -969,7 +947,6 @@
       <c r="F20" s="2" t="n"/>
       <c r="G20" s="2" t="n"/>
       <c r="H20" s="2" t="n"/>
-      <c r="I20" s="2" t="n"/>
     </row>
     <row r="21">
       <c r="A21" s="2" t="n"/>
@@ -980,7 +957,6 @@
       <c r="F21" s="2" t="n"/>
       <c r="G21" s="2" t="n"/>
       <c r="H21" s="2" t="n"/>
-      <c r="I21" s="2" t="n"/>
     </row>
     <row r="22">
       <c r="A22" s="2" t="n"/>
@@ -991,7 +967,6 @@
       <c r="F22" s="2" t="n"/>
       <c r="G22" s="2" t="n"/>
       <c r="H22" s="2" t="n"/>
-      <c r="I22" s="2" t="n"/>
     </row>
     <row r="23">
       <c r="A23" s="2" t="n"/>
@@ -1002,7 +977,6 @@
       <c r="F23" s="2" t="n"/>
       <c r="G23" s="2" t="n"/>
       <c r="H23" s="2" t="n"/>
-      <c r="I23" s="2" t="n"/>
     </row>
     <row r="24">
       <c r="A24" s="2" t="n"/>
@@ -1013,7 +987,6 @@
       <c r="F24" s="2" t="n"/>
       <c r="G24" s="2" t="n"/>
       <c r="H24" s="2" t="n"/>
-      <c r="I24" s="2" t="n"/>
     </row>
     <row r="25">
       <c r="A25" s="2" t="n"/>
@@ -1024,7 +997,6 @@
       <c r="F25" s="2" t="n"/>
       <c r="G25" s="2" t="n"/>
       <c r="H25" s="2" t="n"/>
-      <c r="I25" s="2" t="n"/>
     </row>
     <row r="26">
       <c r="A26" s="2" t="n"/>
@@ -1035,7 +1007,6 @@
       <c r="F26" s="2" t="n"/>
       <c r="G26" s="2" t="n"/>
       <c r="H26" s="2" t="n"/>
-      <c r="I26" s="2" t="n"/>
     </row>
     <row r="27">
       <c r="A27" s="2" t="n"/>
@@ -1046,7 +1017,6 @@
       <c r="F27" s="2" t="n"/>
       <c r="G27" s="2" t="n"/>
       <c r="H27" s="2" t="n"/>
-      <c r="I27" s="2" t="n"/>
     </row>
     <row r="28">
       <c r="A28" s="2" t="n"/>
@@ -1057,7 +1027,6 @@
       <c r="F28" s="2" t="n"/>
       <c r="G28" s="2" t="n"/>
       <c r="H28" s="2" t="n"/>
-      <c r="I28" s="2" t="n"/>
     </row>
     <row r="29">
       <c r="A29" s="2" t="n"/>
@@ -1068,7 +1037,6 @@
       <c r="F29" s="2" t="n"/>
       <c r="G29" s="2" t="n"/>
       <c r="H29" s="2" t="n"/>
-      <c r="I29" s="2" t="n"/>
     </row>
     <row r="30">
       <c r="A30" s="2" t="n"/>
@@ -1079,7 +1047,6 @@
       <c r="F30" s="2" t="n"/>
       <c r="G30" s="2" t="n"/>
       <c r="H30" s="2" t="n"/>
-      <c r="I30" s="2" t="n"/>
     </row>
     <row r="31">
       <c r="A31" s="2" t="n"/>
@@ -1090,7 +1057,6 @@
       <c r="F31" s="2" t="n"/>
       <c r="G31" s="2" t="n"/>
       <c r="H31" s="2" t="n"/>
-      <c r="I31" s="2" t="n"/>
     </row>
     <row r="32">
       <c r="A32" s="2" t="n"/>
@@ -1101,7 +1067,6 @@
       <c r="F32" s="2" t="n"/>
       <c r="G32" s="2" t="n"/>
       <c r="H32" s="2" t="n"/>
-      <c r="I32" s="2" t="n"/>
     </row>
     <row r="33">
       <c r="A33" s="2" t="n"/>
@@ -1112,7 +1077,6 @@
       <c r="F33" s="2" t="n"/>
       <c r="G33" s="2" t="n"/>
       <c r="H33" s="2" t="n"/>
-      <c r="I33" s="2" t="n"/>
     </row>
     <row r="34">
       <c r="A34" s="2" t="n"/>
@@ -1123,7 +1087,6 @@
       <c r="F34" s="2" t="n"/>
       <c r="G34" s="2" t="n"/>
       <c r="H34" s="2" t="n"/>
-      <c r="I34" s="2" t="n"/>
     </row>
     <row r="35">
       <c r="A35" s="2" t="n"/>
@@ -1134,7 +1097,6 @@
       <c r="F35" s="2" t="n"/>
       <c r="G35" s="2" t="n"/>
       <c r="H35" s="2" t="n"/>
-      <c r="I35" s="2" t="n"/>
     </row>
     <row r="36">
       <c r="A36" s="2" t="n"/>
@@ -1145,7 +1107,6 @@
       <c r="F36" s="2" t="n"/>
       <c r="G36" s="2" t="n"/>
       <c r="H36" s="2" t="n"/>
-      <c r="I36" s="2" t="n"/>
     </row>
     <row r="37">
       <c r="A37" s="2" t="n"/>
@@ -1156,7 +1117,6 @@
       <c r="F37" s="2" t="n"/>
       <c r="G37" s="2" t="n"/>
       <c r="H37" s="2" t="n"/>
-      <c r="I37" s="2" t="n"/>
     </row>
     <row r="38">
       <c r="A38" s="2" t="n"/>
@@ -1167,7 +1127,6 @@
       <c r="F38" s="2" t="n"/>
       <c r="G38" s="2" t="n"/>
       <c r="H38" s="2" t="n"/>
-      <c r="I38" s="2" t="n"/>
     </row>
     <row r="39">
       <c r="A39" s="2" t="n"/>
@@ -1178,7 +1137,6 @@
       <c r="F39" s="2" t="n"/>
       <c r="G39" s="2" t="n"/>
       <c r="H39" s="2" t="n"/>
-      <c r="I39" s="2" t="n"/>
     </row>
     <row r="40">
       <c r="A40" s="2" t="n"/>
@@ -1189,7 +1147,6 @@
       <c r="F40" s="2" t="n"/>
       <c r="G40" s="2" t="n"/>
       <c r="H40" s="2" t="n"/>
-      <c r="I40" s="2" t="n"/>
     </row>
     <row r="41">
       <c r="A41" s="2" t="n"/>
@@ -1200,7 +1157,6 @@
       <c r="F41" s="2" t="n"/>
       <c r="G41" s="2" t="n"/>
       <c r="H41" s="2" t="n"/>
-      <c r="I41" s="2" t="n"/>
     </row>
     <row r="42">
       <c r="A42" s="2" t="n"/>
@@ -1211,7 +1167,6 @@
       <c r="F42" s="2" t="n"/>
       <c r="G42" s="2" t="n"/>
       <c r="H42" s="2" t="n"/>
-      <c r="I42" s="2" t="n"/>
     </row>
     <row r="43">
       <c r="A43" s="2" t="n"/>
@@ -1222,7 +1177,6 @@
       <c r="F43" s="2" t="n"/>
       <c r="G43" s="2" t="n"/>
       <c r="H43" s="2" t="n"/>
-      <c r="I43" s="2" t="n"/>
     </row>
     <row r="44">
       <c r="A44" s="2" t="n"/>
@@ -1233,7 +1187,6 @@
       <c r="F44" s="2" t="n"/>
       <c r="G44" s="2" t="n"/>
       <c r="H44" s="2" t="n"/>
-      <c r="I44" s="2" t="n"/>
     </row>
     <row r="45">
       <c r="A45" s="2" t="n"/>
@@ -1244,7 +1197,6 @@
       <c r="F45" s="2" t="n"/>
       <c r="G45" s="2" t="n"/>
       <c r="H45" s="2" t="n"/>
-      <c r="I45" s="2" t="n"/>
     </row>
     <row r="46">
       <c r="A46" s="2" t="n"/>
@@ -1255,7 +1207,6 @@
       <c r="F46" s="2" t="n"/>
       <c r="G46" s="2" t="n"/>
       <c r="H46" s="2" t="n"/>
-      <c r="I46" s="2" t="n"/>
     </row>
     <row r="47">
       <c r="A47" s="2" t="n"/>
@@ -1266,7 +1217,6 @@
       <c r="F47" s="2" t="n"/>
       <c r="G47" s="2" t="n"/>
       <c r="H47" s="2" t="n"/>
-      <c r="I47" s="2" t="n"/>
     </row>
     <row r="48">
       <c r="A48" s="2" t="n"/>
@@ -1277,7 +1227,6 @@
       <c r="F48" s="2" t="n"/>
       <c r="G48" s="2" t="n"/>
       <c r="H48" s="2" t="n"/>
-      <c r="I48" s="2" t="n"/>
     </row>
     <row r="49">
       <c r="A49" s="2" t="n"/>
@@ -1288,7 +1237,6 @@
       <c r="F49" s="2" t="n"/>
       <c r="G49" s="2" t="n"/>
       <c r="H49" s="2" t="n"/>
-      <c r="I49" s="2" t="n"/>
     </row>
     <row r="50">
       <c r="A50" s="2" t="n"/>
@@ -1299,7 +1247,6 @@
       <c r="F50" s="2" t="n"/>
       <c r="G50" s="2" t="n"/>
       <c r="H50" s="2" t="n"/>
-      <c r="I50" s="2" t="n"/>
     </row>
     <row r="51">
       <c r="A51" s="2" t="n"/>
@@ -1310,7 +1257,6 @@
       <c r="F51" s="2" t="n"/>
       <c r="G51" s="2" t="n"/>
       <c r="H51" s="2" t="n"/>
-      <c r="I51" s="2" t="n"/>
     </row>
     <row r="52">
       <c r="A52" s="2" t="n"/>
@@ -1321,7 +1267,6 @@
       <c r="F52" s="2" t="n"/>
       <c r="G52" s="2" t="n"/>
       <c r="H52" s="2" t="n"/>
-      <c r="I52" s="2" t="n"/>
     </row>
     <row r="53">
       <c r="A53" s="2" t="n"/>
@@ -1332,7 +1277,6 @@
       <c r="F53" s="2" t="n"/>
       <c r="G53" s="2" t="n"/>
       <c r="H53" s="2" t="n"/>
-      <c r="I53" s="2" t="n"/>
     </row>
     <row r="54">
       <c r="A54" s="2" t="n"/>
@@ -1343,7 +1287,6 @@
       <c r="F54" s="2" t="n"/>
       <c r="G54" s="2" t="n"/>
       <c r="H54" s="2" t="n"/>
-      <c r="I54" s="2" t="n"/>
     </row>
     <row r="55">
       <c r="A55" s="2" t="n"/>
@@ -1354,7 +1297,6 @@
       <c r="F55" s="2" t="n"/>
       <c r="G55" s="2" t="n"/>
       <c r="H55" s="2" t="n"/>
-      <c r="I55" s="2" t="n"/>
     </row>
     <row r="56">
       <c r="A56" s="2" t="n"/>
@@ -1365,7 +1307,6 @@
       <c r="F56" s="2" t="n"/>
       <c r="G56" s="2" t="n"/>
       <c r="H56" s="2" t="n"/>
-      <c r="I56" s="2" t="n"/>
     </row>
     <row r="57">
       <c r="A57" s="2" t="n"/>
@@ -1376,7 +1317,6 @@
       <c r="F57" s="2" t="n"/>
       <c r="G57" s="2" t="n"/>
       <c r="H57" s="2" t="n"/>
-      <c r="I57" s="2" t="n"/>
     </row>
     <row r="58">
       <c r="A58" s="2" t="n"/>
@@ -1387,7 +1327,6 @@
       <c r="F58" s="2" t="n"/>
       <c r="G58" s="2" t="n"/>
       <c r="H58" s="2" t="n"/>
-      <c r="I58" s="2" t="n"/>
     </row>
     <row r="59">
       <c r="A59" s="2" t="n"/>
@@ -1398,7 +1337,6 @@
       <c r="F59" s="2" t="n"/>
       <c r="G59" s="2" t="n"/>
       <c r="H59" s="2" t="n"/>
-      <c r="I59" s="2" t="n"/>
     </row>
     <row r="60">
       <c r="A60" s="2" t="n"/>
@@ -1409,7 +1347,6 @@
       <c r="F60" s="2" t="n"/>
       <c r="G60" s="2" t="n"/>
       <c r="H60" s="2" t="n"/>
-      <c r="I60" s="2" t="n"/>
     </row>
     <row r="61">
       <c r="A61" s="2" t="n"/>
@@ -1420,7 +1357,6 @@
       <c r="F61" s="2" t="n"/>
       <c r="G61" s="2" t="n"/>
       <c r="H61" s="2" t="n"/>
-      <c r="I61" s="2" t="n"/>
     </row>
     <row r="62">
       <c r="A62" s="2" t="n"/>
@@ -1431,7 +1367,6 @@
       <c r="F62" s="2" t="n"/>
       <c r="G62" s="2" t="n"/>
       <c r="H62" s="2" t="n"/>
-      <c r="I62" s="2" t="n"/>
     </row>
     <row r="63">
       <c r="A63" s="2" t="n"/>
@@ -1442,7 +1377,6 @@
       <c r="F63" s="2" t="n"/>
       <c r="G63" s="2" t="n"/>
       <c r="H63" s="2" t="n"/>
-      <c r="I63" s="2" t="n"/>
     </row>
     <row r="64">
       <c r="A64" s="2" t="n"/>
@@ -1453,7 +1387,6 @@
       <c r="F64" s="2" t="n"/>
       <c r="G64" s="2" t="n"/>
       <c r="H64" s="2" t="n"/>
-      <c r="I64" s="2" t="n"/>
     </row>
     <row r="65">
       <c r="A65" s="2" t="n"/>
@@ -1464,7 +1397,6 @@
       <c r="F65" s="2" t="n"/>
       <c r="G65" s="2" t="n"/>
       <c r="H65" s="2" t="n"/>
-      <c r="I65" s="2" t="n"/>
     </row>
     <row r="66">
       <c r="A66" s="2" t="n"/>
@@ -1475,7 +1407,6 @@
       <c r="F66" s="2" t="n"/>
       <c r="G66" s="2" t="n"/>
       <c r="H66" s="2" t="n"/>
-      <c r="I66" s="2" t="n"/>
     </row>
     <row r="67">
       <c r="A67" s="2" t="n"/>
@@ -1486,7 +1417,6 @@
       <c r="F67" s="2" t="n"/>
       <c r="G67" s="2" t="n"/>
       <c r="H67" s="2" t="n"/>
-      <c r="I67" s="2" t="n"/>
     </row>
     <row r="68">
       <c r="A68" s="2" t="n"/>
@@ -1497,7 +1427,6 @@
       <c r="F68" s="2" t="n"/>
       <c r="G68" s="2" t="n"/>
       <c r="H68" s="2" t="n"/>
-      <c r="I68" s="2" t="n"/>
     </row>
     <row r="69">
       <c r="A69" s="2" t="n"/>
@@ -1508,7 +1437,6 @@
       <c r="F69" s="2" t="n"/>
       <c r="G69" s="2" t="n"/>
       <c r="H69" s="2" t="n"/>
-      <c r="I69" s="2" t="n"/>
     </row>
     <row r="70">
       <c r="A70" s="2" t="n"/>
@@ -1519,7 +1447,6 @@
       <c r="F70" s="2" t="n"/>
       <c r="G70" s="2" t="n"/>
       <c r="H70" s="2" t="n"/>
-      <c r="I70" s="2" t="n"/>
     </row>
     <row r="71">
       <c r="A71" s="2" t="n"/>
@@ -1530,7 +1457,6 @@
       <c r="F71" s="2" t="n"/>
       <c r="G71" s="2" t="n"/>
       <c r="H71" s="2" t="n"/>
-      <c r="I71" s="2" t="n"/>
     </row>
     <row r="72">
       <c r="A72" s="2" t="n"/>
@@ -1541,7 +1467,6 @@
       <c r="F72" s="2" t="n"/>
       <c r="G72" s="2" t="n"/>
       <c r="H72" s="2" t="n"/>
-      <c r="I72" s="2" t="n"/>
     </row>
     <row r="73">
       <c r="A73" s="2" t="n"/>
@@ -1552,7 +1477,6 @@
       <c r="F73" s="2" t="n"/>
       <c r="G73" s="2" t="n"/>
       <c r="H73" s="2" t="n"/>
-      <c r="I73" s="2" t="n"/>
     </row>
     <row r="74">
       <c r="A74" s="2" t="n"/>
@@ -1563,7 +1487,6 @@
       <c r="F74" s="2" t="n"/>
       <c r="G74" s="2" t="n"/>
       <c r="H74" s="2" t="n"/>
-      <c r="I74" s="2" t="n"/>
     </row>
     <row r="75">
       <c r="A75" s="2" t="n"/>
@@ -1574,7 +1497,6 @@
       <c r="F75" s="2" t="n"/>
       <c r="G75" s="2" t="n"/>
       <c r="H75" s="2" t="n"/>
-      <c r="I75" s="2" t="n"/>
     </row>
     <row r="76">
       <c r="A76" s="2" t="n"/>
@@ -1585,7 +1507,6 @@
       <c r="F76" s="2" t="n"/>
       <c r="G76" s="2" t="n"/>
       <c r="H76" s="2" t="n"/>
-      <c r="I76" s="2" t="n"/>
     </row>
     <row r="77">
       <c r="A77" s="2" t="n"/>
@@ -1596,7 +1517,6 @@
       <c r="F77" s="2" t="n"/>
       <c r="G77" s="2" t="n"/>
       <c r="H77" s="2" t="n"/>
-      <c r="I77" s="2" t="n"/>
     </row>
     <row r="78">
       <c r="A78" s="2" t="n"/>
@@ -1607,7 +1527,6 @@
       <c r="F78" s="2" t="n"/>
       <c r="G78" s="2" t="n"/>
       <c r="H78" s="2" t="n"/>
-      <c r="I78" s="2" t="n"/>
     </row>
     <row r="79">
       <c r="A79" s="2" t="n"/>
@@ -1618,7 +1537,6 @@
       <c r="F79" s="2" t="n"/>
       <c r="G79" s="2" t="n"/>
       <c r="H79" s="2" t="n"/>
-      <c r="I79" s="2" t="n"/>
     </row>
     <row r="80">
       <c r="A80" s="2" t="n"/>
@@ -1629,7 +1547,6 @@
       <c r="F80" s="2" t="n"/>
       <c r="G80" s="2" t="n"/>
       <c r="H80" s="2" t="n"/>
-      <c r="I80" s="2" t="n"/>
     </row>
     <row r="81">
       <c r="A81" s="2" t="n"/>
@@ -1640,7 +1557,6 @@
       <c r="F81" s="2" t="n"/>
       <c r="G81" s="2" t="n"/>
       <c r="H81" s="2" t="n"/>
-      <c r="I81" s="2" t="n"/>
     </row>
     <row r="82">
       <c r="A82" s="2" t="n"/>
@@ -1651,7 +1567,6 @@
       <c r="F82" s="2" t="n"/>
       <c r="G82" s="2" t="n"/>
       <c r="H82" s="2" t="n"/>
-      <c r="I82" s="2" t="n"/>
     </row>
     <row r="83">
       <c r="A83" s="2" t="n"/>
@@ -1662,7 +1577,6 @@
       <c r="F83" s="2" t="n"/>
       <c r="G83" s="2" t="n"/>
       <c r="H83" s="2" t="n"/>
-      <c r="I83" s="2" t="n"/>
     </row>
     <row r="84">
       <c r="A84" s="2" t="n"/>
@@ -1673,7 +1587,6 @@
       <c r="F84" s="2" t="n"/>
       <c r="G84" s="2" t="n"/>
       <c r="H84" s="2" t="n"/>
-      <c r="I84" s="2" t="n"/>
     </row>
     <row r="85">
       <c r="A85" s="2" t="n"/>
@@ -1684,7 +1597,6 @@
       <c r="F85" s="2" t="n"/>
       <c r="G85" s="2" t="n"/>
       <c r="H85" s="2" t="n"/>
-      <c r="I85" s="2" t="n"/>
     </row>
     <row r="86">
       <c r="A86" s="2" t="n"/>
@@ -1695,7 +1607,6 @@
       <c r="F86" s="2" t="n"/>
       <c r="G86" s="2" t="n"/>
       <c r="H86" s="2" t="n"/>
-      <c r="I86" s="2" t="n"/>
     </row>
     <row r="87">
       <c r="A87" s="2" t="n"/>
@@ -1706,7 +1617,6 @@
       <c r="F87" s="2" t="n"/>
       <c r="G87" s="2" t="n"/>
       <c r="H87" s="2" t="n"/>
-      <c r="I87" s="2" t="n"/>
     </row>
     <row r="88">
       <c r="A88" s="2" t="n"/>
@@ -1717,14 +1627,13 @@
       <c r="F88" s="2" t="n"/>
       <c r="G88" s="2" t="n"/>
       <c r="H88" s="2" t="n"/>
-      <c r="I88" s="2" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="2">
     <mergeCell ref="B3:E3"/>
     <mergeCell ref="B2:E2"/>
   </mergeCells>
-  <dataValidations count="5">
+  <dataValidations count="4">
     <dataValidation sqref="D9:D88" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"A lot,A little,Not at all"</formula1>
     </dataValidation>
@@ -1737,9 +1646,6 @@
     <dataValidation sqref="H9:H88" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Automate,Augment,Human"</formula1>
     </dataValidation>
-    <dataValidation sqref="I9:I88" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
-      <formula1>"Yes"</formula1>
-    </dataValidation>
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -1751,7 +1657,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I88"/>
+  <dimension ref="A1:H88"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="36" customWidth="1" min="1" max="1"/>
@@ -1762,13 +1668,12 @@
     <col width="14" customWidth="1" min="6" max="6"/>
     <col width="16" customWidth="1" min="7" max="7"/>
     <col width="14" customWidth="1" min="8" max="8"/>
-    <col width="13" customWidth="1" min="9" max="9"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Your week · one row per thing you produced last week, from your calendar, mail and Slack</t>
+          <t>Your week · one row per atomic task from last week, from your calendar, mail and Slack</t>
         </is>
       </c>
     </row>
@@ -1783,7 +1688,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>My guess, before counting: share of tasks a rule or a judge can check</t>
+          <t>My guess, before counting: share of tasks that are verifiable</t>
         </is>
       </c>
       <c r="B3" s="4" t="n"/>
@@ -1791,7 +1696,7 @@
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>Tasks a rule or a judge can check</t>
+          <t>Verifiable tasks</t>
         </is>
       </c>
       <c r="B4" s="5">
@@ -1802,7 +1707,7 @@
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>Hours a rule or a judge can check</t>
+          <t>Verifiable time</t>
         </is>
       </c>
       <c r="B5" s="5">
@@ -1813,7 +1718,7 @@
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>Checkable, with past examples</t>
+          <t>Verifiable, and the data exists</t>
         </is>
       </c>
       <c r="B6" s="5">
@@ -1824,20 +1729,20 @@
     <row r="8" ht="66" customHeight="1">
       <c r="A8" s="6" t="inlineStr">
         <is>
-          <t>Task
+          <t>Atomic task
 (verb + what you produced)</t>
         </is>
       </c>
       <c r="B8" s="6" t="inlineStr">
         <is>
-          <t>Minutes
-last week</t>
+          <t>Time spent
+(minutes)</t>
         </is>
       </c>
       <c r="C8" s="6" t="inlineStr">
         <is>
-          <t>Done right when…
-(what must be true for it to count as done well)</t>
+          <t>Success criteria
+(what must be true for it to count as done)</t>
         </is>
       </c>
       <c r="D8" s="6" t="inlineStr">
@@ -1848,30 +1753,24 @@
       </c>
       <c r="E8" s="6" t="inlineStr">
         <is>
-          <t>Who or what checks it
+          <t>Verifier
 (a rule, or judge · signal · when)</t>
         </is>
       </c>
       <c r="F8" s="6" t="inlineStr">
         <is>
-          <t>Type</t>
+          <t>Verification type</t>
         </is>
       </c>
       <c r="G8" s="6" t="inlineStr">
         <is>
-          <t>Past examples
-(input + correct output)</t>
+          <t>Data
+(past input and output pairs)</t>
         </is>
       </c>
       <c r="H8" s="6" t="inlineStr">
         <is>
           <t>Bucket</t>
-        </is>
-      </c>
-      <c r="I8" s="6" t="inlineStr">
-        <is>
-          <t>Build a model for this?
-(pick one)</t>
         </is>
       </c>
     </row>
@@ -1884,7 +1783,6 @@
       <c r="F9" s="2" t="n"/>
       <c r="G9" s="2" t="n"/>
       <c r="H9" s="2" t="n"/>
-      <c r="I9" s="2" t="n"/>
     </row>
     <row r="10">
       <c r="A10" s="2" t="n"/>
@@ -1895,7 +1793,6 @@
       <c r="F10" s="2" t="n"/>
       <c r="G10" s="2" t="n"/>
       <c r="H10" s="2" t="n"/>
-      <c r="I10" s="2" t="n"/>
     </row>
     <row r="11">
       <c r="A11" s="2" t="n"/>
@@ -1906,7 +1803,6 @@
       <c r="F11" s="2" t="n"/>
       <c r="G11" s="2" t="n"/>
       <c r="H11" s="2" t="n"/>
-      <c r="I11" s="2" t="n"/>
     </row>
     <row r="12">
       <c r="A12" s="2" t="n"/>
@@ -1917,7 +1813,6 @@
       <c r="F12" s="2" t="n"/>
       <c r="G12" s="2" t="n"/>
       <c r="H12" s="2" t="n"/>
-      <c r="I12" s="2" t="n"/>
     </row>
     <row r="13">
       <c r="A13" s="2" t="n"/>
@@ -1928,7 +1823,6 @@
       <c r="F13" s="2" t="n"/>
       <c r="G13" s="2" t="n"/>
       <c r="H13" s="2" t="n"/>
-      <c r="I13" s="2" t="n"/>
     </row>
     <row r="14">
       <c r="A14" s="2" t="n"/>
@@ -1939,7 +1833,6 @@
       <c r="F14" s="2" t="n"/>
       <c r="G14" s="2" t="n"/>
       <c r="H14" s="2" t="n"/>
-      <c r="I14" s="2" t="n"/>
     </row>
     <row r="15">
       <c r="A15" s="2" t="n"/>
@@ -1950,7 +1843,6 @@
       <c r="F15" s="2" t="n"/>
       <c r="G15" s="2" t="n"/>
       <c r="H15" s="2" t="n"/>
-      <c r="I15" s="2" t="n"/>
     </row>
     <row r="16">
       <c r="A16" s="2" t="n"/>
@@ -1961,7 +1853,6 @@
       <c r="F16" s="2" t="n"/>
       <c r="G16" s="2" t="n"/>
       <c r="H16" s="2" t="n"/>
-      <c r="I16" s="2" t="n"/>
     </row>
     <row r="17">
       <c r="A17" s="2" t="n"/>
@@ -1972,7 +1863,6 @@
       <c r="F17" s="2" t="n"/>
       <c r="G17" s="2" t="n"/>
       <c r="H17" s="2" t="n"/>
-      <c r="I17" s="2" t="n"/>
     </row>
     <row r="18">
       <c r="A18" s="2" t="n"/>
@@ -1983,7 +1873,6 @@
       <c r="F18" s="2" t="n"/>
       <c r="G18" s="2" t="n"/>
       <c r="H18" s="2" t="n"/>
-      <c r="I18" s="2" t="n"/>
     </row>
     <row r="19">
       <c r="A19" s="2" t="n"/>
@@ -1994,7 +1883,6 @@
       <c r="F19" s="2" t="n"/>
       <c r="G19" s="2" t="n"/>
       <c r="H19" s="2" t="n"/>
-      <c r="I19" s="2" t="n"/>
     </row>
     <row r="20">
       <c r="A20" s="2" t="n"/>
@@ -2005,7 +1893,6 @@
       <c r="F20" s="2" t="n"/>
       <c r="G20" s="2" t="n"/>
       <c r="H20" s="2" t="n"/>
-      <c r="I20" s="2" t="n"/>
     </row>
     <row r="21">
       <c r="A21" s="2" t="n"/>
@@ -2016,7 +1903,6 @@
       <c r="F21" s="2" t="n"/>
       <c r="G21" s="2" t="n"/>
       <c r="H21" s="2" t="n"/>
-      <c r="I21" s="2" t="n"/>
     </row>
     <row r="22">
       <c r="A22" s="2" t="n"/>
@@ -2027,7 +1913,6 @@
       <c r="F22" s="2" t="n"/>
       <c r="G22" s="2" t="n"/>
       <c r="H22" s="2" t="n"/>
-      <c r="I22" s="2" t="n"/>
     </row>
     <row r="23">
       <c r="A23" s="2" t="n"/>
@@ -2038,7 +1923,6 @@
       <c r="F23" s="2" t="n"/>
       <c r="G23" s="2" t="n"/>
       <c r="H23" s="2" t="n"/>
-      <c r="I23" s="2" t="n"/>
     </row>
     <row r="24">
       <c r="A24" s="2" t="n"/>
@@ -2049,7 +1933,6 @@
       <c r="F24" s="2" t="n"/>
       <c r="G24" s="2" t="n"/>
       <c r="H24" s="2" t="n"/>
-      <c r="I24" s="2" t="n"/>
     </row>
     <row r="25">
       <c r="A25" s="2" t="n"/>
@@ -2060,7 +1943,6 @@
       <c r="F25" s="2" t="n"/>
       <c r="G25" s="2" t="n"/>
       <c r="H25" s="2" t="n"/>
-      <c r="I25" s="2" t="n"/>
     </row>
     <row r="26">
       <c r="A26" s="2" t="n"/>
@@ -2071,7 +1953,6 @@
       <c r="F26" s="2" t="n"/>
       <c r="G26" s="2" t="n"/>
       <c r="H26" s="2" t="n"/>
-      <c r="I26" s="2" t="n"/>
     </row>
     <row r="27">
       <c r="A27" s="2" t="n"/>
@@ -2082,7 +1963,6 @@
       <c r="F27" s="2" t="n"/>
       <c r="G27" s="2" t="n"/>
       <c r="H27" s="2" t="n"/>
-      <c r="I27" s="2" t="n"/>
     </row>
     <row r="28">
       <c r="A28" s="2" t="n"/>
@@ -2093,7 +1973,6 @@
       <c r="F28" s="2" t="n"/>
       <c r="G28" s="2" t="n"/>
       <c r="H28" s="2" t="n"/>
-      <c r="I28" s="2" t="n"/>
     </row>
     <row r="29">
       <c r="A29" s="2" t="n"/>
@@ -2104,7 +1983,6 @@
       <c r="F29" s="2" t="n"/>
       <c r="G29" s="2" t="n"/>
       <c r="H29" s="2" t="n"/>
-      <c r="I29" s="2" t="n"/>
     </row>
     <row r="30">
       <c r="A30" s="2" t="n"/>
@@ -2115,7 +1993,6 @@
       <c r="F30" s="2" t="n"/>
       <c r="G30" s="2" t="n"/>
       <c r="H30" s="2" t="n"/>
-      <c r="I30" s="2" t="n"/>
     </row>
     <row r="31">
       <c r="A31" s="2" t="n"/>
@@ -2126,7 +2003,6 @@
       <c r="F31" s="2" t="n"/>
       <c r="G31" s="2" t="n"/>
       <c r="H31" s="2" t="n"/>
-      <c r="I31" s="2" t="n"/>
     </row>
     <row r="32">
       <c r="A32" s="2" t="n"/>
@@ -2137,7 +2013,6 @@
       <c r="F32" s="2" t="n"/>
       <c r="G32" s="2" t="n"/>
       <c r="H32" s="2" t="n"/>
-      <c r="I32" s="2" t="n"/>
     </row>
     <row r="33">
       <c r="A33" s="2" t="n"/>
@@ -2148,7 +2023,6 @@
       <c r="F33" s="2" t="n"/>
       <c r="G33" s="2" t="n"/>
       <c r="H33" s="2" t="n"/>
-      <c r="I33" s="2" t="n"/>
     </row>
     <row r="34">
       <c r="A34" s="2" t="n"/>
@@ -2159,7 +2033,6 @@
       <c r="F34" s="2" t="n"/>
       <c r="G34" s="2" t="n"/>
       <c r="H34" s="2" t="n"/>
-      <c r="I34" s="2" t="n"/>
     </row>
     <row r="35">
       <c r="A35" s="2" t="n"/>
@@ -2170,7 +2043,6 @@
       <c r="F35" s="2" t="n"/>
       <c r="G35" s="2" t="n"/>
       <c r="H35" s="2" t="n"/>
-      <c r="I35" s="2" t="n"/>
     </row>
     <row r="36">
       <c r="A36" s="2" t="n"/>
@@ -2181,7 +2053,6 @@
       <c r="F36" s="2" t="n"/>
       <c r="G36" s="2" t="n"/>
       <c r="H36" s="2" t="n"/>
-      <c r="I36" s="2" t="n"/>
     </row>
     <row r="37">
       <c r="A37" s="2" t="n"/>
@@ -2192,7 +2063,6 @@
       <c r="F37" s="2" t="n"/>
       <c r="G37" s="2" t="n"/>
       <c r="H37" s="2" t="n"/>
-      <c r="I37" s="2" t="n"/>
     </row>
     <row r="38">
       <c r="A38" s="2" t="n"/>
@@ -2203,7 +2073,6 @@
       <c r="F38" s="2" t="n"/>
       <c r="G38" s="2" t="n"/>
       <c r="H38" s="2" t="n"/>
-      <c r="I38" s="2" t="n"/>
     </row>
     <row r="39">
       <c r="A39" s="2" t="n"/>
@@ -2214,7 +2083,6 @@
       <c r="F39" s="2" t="n"/>
       <c r="G39" s="2" t="n"/>
       <c r="H39" s="2" t="n"/>
-      <c r="I39" s="2" t="n"/>
     </row>
     <row r="40">
       <c r="A40" s="2" t="n"/>
@@ -2225,7 +2093,6 @@
       <c r="F40" s="2" t="n"/>
       <c r="G40" s="2" t="n"/>
       <c r="H40" s="2" t="n"/>
-      <c r="I40" s="2" t="n"/>
     </row>
     <row r="41">
       <c r="A41" s="2" t="n"/>
@@ -2236,7 +2103,6 @@
       <c r="F41" s="2" t="n"/>
       <c r="G41" s="2" t="n"/>
       <c r="H41" s="2" t="n"/>
-      <c r="I41" s="2" t="n"/>
     </row>
     <row r="42">
       <c r="A42" s="2" t="n"/>
@@ -2247,7 +2113,6 @@
       <c r="F42" s="2" t="n"/>
       <c r="G42" s="2" t="n"/>
       <c r="H42" s="2" t="n"/>
-      <c r="I42" s="2" t="n"/>
     </row>
     <row r="43">
       <c r="A43" s="2" t="n"/>
@@ -2258,7 +2123,6 @@
       <c r="F43" s="2" t="n"/>
       <c r="G43" s="2" t="n"/>
       <c r="H43" s="2" t="n"/>
-      <c r="I43" s="2" t="n"/>
     </row>
     <row r="44">
       <c r="A44" s="2" t="n"/>
@@ -2269,7 +2133,6 @@
       <c r="F44" s="2" t="n"/>
       <c r="G44" s="2" t="n"/>
       <c r="H44" s="2" t="n"/>
-      <c r="I44" s="2" t="n"/>
     </row>
     <row r="45">
       <c r="A45" s="2" t="n"/>
@@ -2280,7 +2143,6 @@
       <c r="F45" s="2" t="n"/>
       <c r="G45" s="2" t="n"/>
       <c r="H45" s="2" t="n"/>
-      <c r="I45" s="2" t="n"/>
     </row>
     <row r="46">
       <c r="A46" s="2" t="n"/>
@@ -2291,7 +2153,6 @@
       <c r="F46" s="2" t="n"/>
       <c r="G46" s="2" t="n"/>
       <c r="H46" s="2" t="n"/>
-      <c r="I46" s="2" t="n"/>
     </row>
     <row r="47">
       <c r="A47" s="2" t="n"/>
@@ -2302,7 +2163,6 @@
       <c r="F47" s="2" t="n"/>
       <c r="G47" s="2" t="n"/>
       <c r="H47" s="2" t="n"/>
-      <c r="I47" s="2" t="n"/>
     </row>
     <row r="48">
       <c r="A48" s="2" t="n"/>
@@ -2313,7 +2173,6 @@
       <c r="F48" s="2" t="n"/>
       <c r="G48" s="2" t="n"/>
       <c r="H48" s="2" t="n"/>
-      <c r="I48" s="2" t="n"/>
     </row>
     <row r="49">
       <c r="A49" s="2" t="n"/>
@@ -2324,7 +2183,6 @@
       <c r="F49" s="2" t="n"/>
       <c r="G49" s="2" t="n"/>
       <c r="H49" s="2" t="n"/>
-      <c r="I49" s="2" t="n"/>
     </row>
     <row r="50">
       <c r="A50" s="2" t="n"/>
@@ -2335,7 +2193,6 @@
       <c r="F50" s="2" t="n"/>
       <c r="G50" s="2" t="n"/>
       <c r="H50" s="2" t="n"/>
-      <c r="I50" s="2" t="n"/>
     </row>
     <row r="51">
       <c r="A51" s="2" t="n"/>
@@ -2346,7 +2203,6 @@
       <c r="F51" s="2" t="n"/>
       <c r="G51" s="2" t="n"/>
       <c r="H51" s="2" t="n"/>
-      <c r="I51" s="2" t="n"/>
     </row>
     <row r="52">
       <c r="A52" s="2" t="n"/>
@@ -2357,7 +2213,6 @@
       <c r="F52" s="2" t="n"/>
       <c r="G52" s="2" t="n"/>
       <c r="H52" s="2" t="n"/>
-      <c r="I52" s="2" t="n"/>
     </row>
     <row r="53">
       <c r="A53" s="2" t="n"/>
@@ -2368,7 +2223,6 @@
       <c r="F53" s="2" t="n"/>
       <c r="G53" s="2" t="n"/>
       <c r="H53" s="2" t="n"/>
-      <c r="I53" s="2" t="n"/>
     </row>
     <row r="54">
       <c r="A54" s="2" t="n"/>
@@ -2379,7 +2233,6 @@
       <c r="F54" s="2" t="n"/>
       <c r="G54" s="2" t="n"/>
       <c r="H54" s="2" t="n"/>
-      <c r="I54" s="2" t="n"/>
     </row>
     <row r="55">
       <c r="A55" s="2" t="n"/>
@@ -2390,7 +2243,6 @@
       <c r="F55" s="2" t="n"/>
       <c r="G55" s="2" t="n"/>
       <c r="H55" s="2" t="n"/>
-      <c r="I55" s="2" t="n"/>
     </row>
     <row r="56">
       <c r="A56" s="2" t="n"/>
@@ -2401,7 +2253,6 @@
       <c r="F56" s="2" t="n"/>
       <c r="G56" s="2" t="n"/>
       <c r="H56" s="2" t="n"/>
-      <c r="I56" s="2" t="n"/>
     </row>
     <row r="57">
       <c r="A57" s="2" t="n"/>
@@ -2412,7 +2263,6 @@
       <c r="F57" s="2" t="n"/>
       <c r="G57" s="2" t="n"/>
       <c r="H57" s="2" t="n"/>
-      <c r="I57" s="2" t="n"/>
     </row>
     <row r="58">
       <c r="A58" s="2" t="n"/>
@@ -2423,7 +2273,6 @@
       <c r="F58" s="2" t="n"/>
       <c r="G58" s="2" t="n"/>
       <c r="H58" s="2" t="n"/>
-      <c r="I58" s="2" t="n"/>
     </row>
     <row r="59">
       <c r="A59" s="2" t="n"/>
@@ -2434,7 +2283,6 @@
       <c r="F59" s="2" t="n"/>
       <c r="G59" s="2" t="n"/>
       <c r="H59" s="2" t="n"/>
-      <c r="I59" s="2" t="n"/>
     </row>
     <row r="60">
       <c r="A60" s="2" t="n"/>
@@ -2445,7 +2293,6 @@
       <c r="F60" s="2" t="n"/>
       <c r="G60" s="2" t="n"/>
       <c r="H60" s="2" t="n"/>
-      <c r="I60" s="2" t="n"/>
     </row>
     <row r="61">
       <c r="A61" s="2" t="n"/>
@@ -2456,7 +2303,6 @@
       <c r="F61" s="2" t="n"/>
       <c r="G61" s="2" t="n"/>
       <c r="H61" s="2" t="n"/>
-      <c r="I61" s="2" t="n"/>
     </row>
     <row r="62">
       <c r="A62" s="2" t="n"/>
@@ -2467,7 +2313,6 @@
       <c r="F62" s="2" t="n"/>
       <c r="G62" s="2" t="n"/>
       <c r="H62" s="2" t="n"/>
-      <c r="I62" s="2" t="n"/>
     </row>
     <row r="63">
       <c r="A63" s="2" t="n"/>
@@ -2478,7 +2323,6 @@
       <c r="F63" s="2" t="n"/>
       <c r="G63" s="2" t="n"/>
       <c r="H63" s="2" t="n"/>
-      <c r="I63" s="2" t="n"/>
     </row>
     <row r="64">
       <c r="A64" s="2" t="n"/>
@@ -2489,7 +2333,6 @@
       <c r="F64" s="2" t="n"/>
       <c r="G64" s="2" t="n"/>
       <c r="H64" s="2" t="n"/>
-      <c r="I64" s="2" t="n"/>
     </row>
     <row r="65">
       <c r="A65" s="2" t="n"/>
@@ -2500,7 +2343,6 @@
       <c r="F65" s="2" t="n"/>
       <c r="G65" s="2" t="n"/>
       <c r="H65" s="2" t="n"/>
-      <c r="I65" s="2" t="n"/>
     </row>
     <row r="66">
       <c r="A66" s="2" t="n"/>
@@ -2511,7 +2353,6 @@
       <c r="F66" s="2" t="n"/>
       <c r="G66" s="2" t="n"/>
       <c r="H66" s="2" t="n"/>
-      <c r="I66" s="2" t="n"/>
     </row>
     <row r="67">
       <c r="A67" s="2" t="n"/>
@@ -2522,7 +2363,6 @@
       <c r="F67" s="2" t="n"/>
       <c r="G67" s="2" t="n"/>
       <c r="H67" s="2" t="n"/>
-      <c r="I67" s="2" t="n"/>
     </row>
     <row r="68">
       <c r="A68" s="2" t="n"/>
@@ -2533,7 +2373,6 @@
       <c r="F68" s="2" t="n"/>
       <c r="G68" s="2" t="n"/>
       <c r="H68" s="2" t="n"/>
-      <c r="I68" s="2" t="n"/>
     </row>
     <row r="69">
       <c r="A69" s="2" t="n"/>
@@ -2544,7 +2383,6 @@
       <c r="F69" s="2" t="n"/>
       <c r="G69" s="2" t="n"/>
       <c r="H69" s="2" t="n"/>
-      <c r="I69" s="2" t="n"/>
     </row>
     <row r="70">
       <c r="A70" s="2" t="n"/>
@@ -2555,7 +2393,6 @@
       <c r="F70" s="2" t="n"/>
       <c r="G70" s="2" t="n"/>
       <c r="H70" s="2" t="n"/>
-      <c r="I70" s="2" t="n"/>
     </row>
     <row r="71">
       <c r="A71" s="2" t="n"/>
@@ -2566,7 +2403,6 @@
       <c r="F71" s="2" t="n"/>
       <c r="G71" s="2" t="n"/>
       <c r="H71" s="2" t="n"/>
-      <c r="I71" s="2" t="n"/>
     </row>
     <row r="72">
       <c r="A72" s="2" t="n"/>
@@ -2577,7 +2413,6 @@
       <c r="F72" s="2" t="n"/>
       <c r="G72" s="2" t="n"/>
       <c r="H72" s="2" t="n"/>
-      <c r="I72" s="2" t="n"/>
     </row>
     <row r="73">
       <c r="A73" s="2" t="n"/>
@@ -2588,7 +2423,6 @@
       <c r="F73" s="2" t="n"/>
       <c r="G73" s="2" t="n"/>
       <c r="H73" s="2" t="n"/>
-      <c r="I73" s="2" t="n"/>
     </row>
     <row r="74">
       <c r="A74" s="2" t="n"/>
@@ -2599,7 +2433,6 @@
       <c r="F74" s="2" t="n"/>
       <c r="G74" s="2" t="n"/>
       <c r="H74" s="2" t="n"/>
-      <c r="I74" s="2" t="n"/>
     </row>
     <row r="75">
       <c r="A75" s="2" t="n"/>
@@ -2610,7 +2443,6 @@
       <c r="F75" s="2" t="n"/>
       <c r="G75" s="2" t="n"/>
       <c r="H75" s="2" t="n"/>
-      <c r="I75" s="2" t="n"/>
     </row>
     <row r="76">
       <c r="A76" s="2" t="n"/>
@@ -2621,7 +2453,6 @@
       <c r="F76" s="2" t="n"/>
       <c r="G76" s="2" t="n"/>
       <c r="H76" s="2" t="n"/>
-      <c r="I76" s="2" t="n"/>
     </row>
     <row r="77">
       <c r="A77" s="2" t="n"/>
@@ -2632,7 +2463,6 @@
       <c r="F77" s="2" t="n"/>
       <c r="G77" s="2" t="n"/>
       <c r="H77" s="2" t="n"/>
-      <c r="I77" s="2" t="n"/>
     </row>
     <row r="78">
       <c r="A78" s="2" t="n"/>
@@ -2643,7 +2473,6 @@
       <c r="F78" s="2" t="n"/>
       <c r="G78" s="2" t="n"/>
       <c r="H78" s="2" t="n"/>
-      <c r="I78" s="2" t="n"/>
     </row>
     <row r="79">
       <c r="A79" s="2" t="n"/>
@@ -2654,7 +2483,6 @@
       <c r="F79" s="2" t="n"/>
       <c r="G79" s="2" t="n"/>
       <c r="H79" s="2" t="n"/>
-      <c r="I79" s="2" t="n"/>
     </row>
     <row r="80">
       <c r="A80" s="2" t="n"/>
@@ -2665,7 +2493,6 @@
       <c r="F80" s="2" t="n"/>
       <c r="G80" s="2" t="n"/>
       <c r="H80" s="2" t="n"/>
-      <c r="I80" s="2" t="n"/>
     </row>
     <row r="81">
       <c r="A81" s="2" t="n"/>
@@ -2676,7 +2503,6 @@
       <c r="F81" s="2" t="n"/>
       <c r="G81" s="2" t="n"/>
       <c r="H81" s="2" t="n"/>
-      <c r="I81" s="2" t="n"/>
     </row>
     <row r="82">
       <c r="A82" s="2" t="n"/>
@@ -2687,7 +2513,6 @@
       <c r="F82" s="2" t="n"/>
       <c r="G82" s="2" t="n"/>
       <c r="H82" s="2" t="n"/>
-      <c r="I82" s="2" t="n"/>
     </row>
     <row r="83">
       <c r="A83" s="2" t="n"/>
@@ -2698,7 +2523,6 @@
       <c r="F83" s="2" t="n"/>
       <c r="G83" s="2" t="n"/>
       <c r="H83" s="2" t="n"/>
-      <c r="I83" s="2" t="n"/>
     </row>
     <row r="84">
       <c r="A84" s="2" t="n"/>
@@ -2709,7 +2533,6 @@
       <c r="F84" s="2" t="n"/>
       <c r="G84" s="2" t="n"/>
       <c r="H84" s="2" t="n"/>
-      <c r="I84" s="2" t="n"/>
     </row>
     <row r="85">
       <c r="A85" s="2" t="n"/>
@@ -2720,7 +2543,6 @@
       <c r="F85" s="2" t="n"/>
       <c r="G85" s="2" t="n"/>
       <c r="H85" s="2" t="n"/>
-      <c r="I85" s="2" t="n"/>
     </row>
     <row r="86">
       <c r="A86" s="2" t="n"/>
@@ -2731,7 +2553,6 @@
       <c r="F86" s="2" t="n"/>
       <c r="G86" s="2" t="n"/>
       <c r="H86" s="2" t="n"/>
-      <c r="I86" s="2" t="n"/>
     </row>
     <row r="87">
       <c r="A87" s="2" t="n"/>
@@ -2742,7 +2563,6 @@
       <c r="F87" s="2" t="n"/>
       <c r="G87" s="2" t="n"/>
       <c r="H87" s="2" t="n"/>
-      <c r="I87" s="2" t="n"/>
     </row>
     <row r="88">
       <c r="A88" s="2" t="n"/>
@@ -2753,14 +2573,13 @@
       <c r="F88" s="2" t="n"/>
       <c r="G88" s="2" t="n"/>
       <c r="H88" s="2" t="n"/>
-      <c r="I88" s="2" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="2">
     <mergeCell ref="B3:E3"/>
     <mergeCell ref="B2:E2"/>
   </mergeCells>
-  <dataValidations count="5">
+  <dataValidations count="4">
     <dataValidation sqref="D9:D88" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"A lot,A little,Not at all"</formula1>
     </dataValidation>
@@ -2773,9 +2592,6 @@
     <dataValidation sqref="H9:H88" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Automate,Augment,Human"</formula1>
     </dataValidation>
-    <dataValidation sqref="I9:I88" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
-      <formula1>"Yes"</formula1>
-    </dataValidation>
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Lecture 9 practice set: Unverifiable as the third verification type
The sheet's dropdown, its formulas and Aarav's CFO row use Unverifiable; the
page names all three verification types and points the bucket step at Rules.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/_plan/l09-template/verify-your-own-job-template.xlsx
+++ b/_plan/l09-template/verify-your-own-job-template.xlsx
@@ -459,7 +459,7 @@
     <col width="34" customWidth="1" min="3" max="3"/>
     <col width="17" customWidth="1" min="4" max="4"/>
     <col width="44" customWidth="1" min="5" max="5"/>
-    <col width="14" customWidth="1" min="6" max="6"/>
+    <col width="17" customWidth="1" min="6" max="6"/>
     <col width="16" customWidth="1" min="7" max="7"/>
     <col width="14" customWidth="1" min="8" max="8"/>
   </cols>
@@ -500,7 +500,7 @@
         </is>
       </c>
       <c r="B4" s="5">
-        <f>IFERROR((COUNTIF(F9:F88,"Rule")+COUNTIF(F9:F88,"Judgment"))/(COUNTIF(F9:F88,"Rule")+COUNTIF(F9:F88,"Judgment")+COUNTIF(F9:F88,"None")),"")</f>
+        <f>IFERROR((COUNTIF(F9:F88,"Rule")+COUNTIF(F9:F88,"Judgment"))/(COUNTIF(F9:F88,"Rule")+COUNTIF(F9:F88,"Judgment")+COUNTIF(F9:F88,"Unverifiable")),"")</f>
         <v/>
       </c>
     </row>
@@ -522,7 +522,7 @@
         </is>
       </c>
       <c r="B6" s="5">
-        <f>IFERROR((COUNTIFS(F9:F88,"Rule",G9:G88,"&lt;&gt;None",G9:G88,"&lt;&gt;")+COUNTIFS(F9:F88,"Judgment",G9:G88,"&lt;&gt;None",G9:G88,"&lt;&gt;"))/(COUNTIF(F9:F88,"Rule")+COUNTIF(F9:F88,"Judgment")+COUNTIF(F9:F88,"None")),"")</f>
+        <f>IFERROR((COUNTIFS(F9:F88,"Rule",G9:G88,"&lt;&gt;None",G9:G88,"&lt;&gt;")+COUNTIFS(F9:F88,"Judgment",G9:G88,"&lt;&gt;None",G9:G88,"&lt;&gt;"))/(COUNTIF(F9:F88,"Rule")+COUNTIF(F9:F88,"Judgment")+COUNTIF(F9:F88,"Unverifiable")),"")</f>
         <v/>
       </c>
     </row>
@@ -904,7 +904,7 @@
       </c>
       <c r="F17" s="2" t="inlineStr">
         <is>
-          <t>None</t>
+          <t>Unverifiable</t>
         </is>
       </c>
       <c r="G17" s="2" t="inlineStr">
@@ -1638,7 +1638,7 @@
       <formula1>"A lot,A little,Not at all"</formula1>
     </dataValidation>
     <dataValidation sqref="F9:F88" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
-      <formula1>"Rule,Judgment,None"</formula1>
+      <formula1>"Rule,Judgment,Unverifiable"</formula1>
     </dataValidation>
     <dataValidation sqref="G9:G88" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"None,Under 10,10 to 100,Over 100"</formula1>
@@ -1665,7 +1665,7 @@
     <col width="34" customWidth="1" min="3" max="3"/>
     <col width="17" customWidth="1" min="4" max="4"/>
     <col width="44" customWidth="1" min="5" max="5"/>
-    <col width="14" customWidth="1" min="6" max="6"/>
+    <col width="17" customWidth="1" min="6" max="6"/>
     <col width="16" customWidth="1" min="7" max="7"/>
     <col width="14" customWidth="1" min="8" max="8"/>
   </cols>
@@ -1700,7 +1700,7 @@
         </is>
       </c>
       <c r="B4" s="5">
-        <f>IFERROR((COUNTIF(F9:F88,"Rule")+COUNTIF(F9:F88,"Judgment"))/(COUNTIF(F9:F88,"Rule")+COUNTIF(F9:F88,"Judgment")+COUNTIF(F9:F88,"None")),"")</f>
+        <f>IFERROR((COUNTIF(F9:F88,"Rule")+COUNTIF(F9:F88,"Judgment"))/(COUNTIF(F9:F88,"Rule")+COUNTIF(F9:F88,"Judgment")+COUNTIF(F9:F88,"Unverifiable")),"")</f>
         <v/>
       </c>
     </row>
@@ -1722,7 +1722,7 @@
         </is>
       </c>
       <c r="B6" s="5">
-        <f>IFERROR((COUNTIFS(F9:F88,"Rule",G9:G88,"&lt;&gt;None",G9:G88,"&lt;&gt;")+COUNTIFS(F9:F88,"Judgment",G9:G88,"&lt;&gt;None",G9:G88,"&lt;&gt;"))/(COUNTIF(F9:F88,"Rule")+COUNTIF(F9:F88,"Judgment")+COUNTIF(F9:F88,"None")),"")</f>
+        <f>IFERROR((COUNTIFS(F9:F88,"Rule",G9:G88,"&lt;&gt;None",G9:G88,"&lt;&gt;")+COUNTIFS(F9:F88,"Judgment",G9:G88,"&lt;&gt;None",G9:G88,"&lt;&gt;"))/(COUNTIF(F9:F88,"Rule")+COUNTIF(F9:F88,"Judgment")+COUNTIF(F9:F88,"Unverifiable")),"")</f>
         <v/>
       </c>
     </row>
@@ -2584,7 +2584,7 @@
       <formula1>"A lot,A little,Not at all"</formula1>
     </dataValidation>
     <dataValidation sqref="F9:F88" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
-      <formula1>"Rule,Judgment,None"</formula1>
+      <formula1>"Rule,Judgment,Unverifiable"</formula1>
     </dataValidation>
     <dataValidation sqref="G9:G88" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"None,Under 10,10 to 100,Over 100"</formula1>

</xml_diff>